<commit_message>
Matchmaker context, doping en admin structuur bijgewerkt
</commit_message>
<xml_diff>
--- a/public/templates/fightsupport-aanmeldingen-upload.xlsx
+++ b/public/templates/fightsupport-aanmeldingen-upload.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\App\Fightsupport\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Apps\Fightsupport\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C063E58-0320-48A8-8E64-A4EDBC2928D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBD04A36-506F-4FFB-892F-A5FAFF64075D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{729028DD-135B-4EB2-BD2B-100D9B9B9271}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{729028DD-135B-4EB2-BD2B-100D9B9B9271}"/>
   </bookViews>
   <sheets>
     <sheet name="Upload aanmeldingen" sheetId="1" r:id="rId1"/>
@@ -29,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Klasse</t>
   </si>
@@ -64,6 +67,9 @@
   </si>
   <si>
     <t xml:space="preserve">KG </t>
+  </si>
+  <si>
+    <t>Geslacht</t>
   </si>
 </sst>
 </file>
@@ -232,8 +238,8 @@
       <xdr:rowOff>22860</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1844040</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1132840</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
@@ -594,37 +600,38 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{848D0188-C820-4E97-A405-5753A30365E6}">
-  <dimension ref="A2:G49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:H49"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="8.453125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1796875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="31.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.81640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E2" s="3" t="s">
+    <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.4">
+      <c r="F2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="9"/>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E3" s="3" t="s">
+      <c r="G2" s="9"/>
+    </row>
+    <row r="3" spans="1:8" ht="16" x14ac:dyDescent="0.4">
+      <c r="F3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="10"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E4" s="11" t="s">
+      <c r="G3" s="10"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="6" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G4" s="2"/>
+    </row>
+    <row r="6" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
@@ -634,196 +641,242 @@
       <c r="C6" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="F6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="7"/>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
-      <c r="F7" s="7"/>
+      <c r="D7" s="7"/>
       <c r="G7" s="7"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7" s="7"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="7"/>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D8" s="7"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D9" s="7"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="7"/>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D10" s="7"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="7"/>
       <c r="B11" s="7"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D11" s="7"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="7"/>
       <c r="B12" s="7"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D12" s="7"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D13" s="7"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D14" s="7"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="7"/>
       <c r="B15" s="7"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D15" s="7"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="7"/>
       <c r="B16" s="7"/>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D16" s="7"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="7"/>
       <c r="B17" s="7"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D17" s="7"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D18" s="7"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D19" s="7"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D20" s="7"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D21" s="7"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D22" s="7"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D23" s="7"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D24" s="7"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="7"/>
       <c r="B25" s="7"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D25" s="7"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="7"/>
       <c r="B26" s="7"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D26" s="7"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="7"/>
       <c r="B27" s="7"/>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D27" s="7"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="7"/>
       <c r="B28" s="7"/>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D28" s="7"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="7"/>
       <c r="B29" s="7"/>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D29" s="7"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="7"/>
       <c r="B30" s="7"/>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D30" s="7"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="7"/>
       <c r="B31" s="7"/>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D31" s="7"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="7"/>
       <c r="B32" s="7"/>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D32" s="7"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="7"/>
       <c r="B33" s="7"/>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D33" s="7"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="7"/>
       <c r="B34" s="7"/>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D34" s="7"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="7"/>
       <c r="B35" s="7"/>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D35" s="7"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="7"/>
       <c r="B36" s="7"/>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D36" s="7"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="7"/>
       <c r="B37" s="7"/>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D37" s="7"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="7"/>
       <c r="B38" s="7"/>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D38" s="7"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D39" s="7"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="7"/>
       <c r="B40" s="7"/>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D40" s="7"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="7"/>
       <c r="B41" s="7"/>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D41" s="7"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="7"/>
       <c r="B42" s="7"/>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D42" s="7"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D43" s="7"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D44" s="7"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D45" s="7"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="7"/>
       <c r="B46" s="7"/>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D46" s="7"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="7"/>
       <c r="B47" s="7"/>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D47" s="7"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D48" s="7"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="7"/>
       <c r="B49" s="7"/>
+      <c r="D49" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>